<commit_message>
chore: T01/T02 改 Neon 連線版 + 清 T07 全部遺留
- T01/T02：DB 從本地 Docker 改連 Neon 雲端（名稱/交付物/備注 + 甘特同步）
- 說明與原則：原則 4/5 更新為 CSV 解耦版，移除「全員玩 Embedding」
- 人力配置：七人任務清單去 T07、任務數 -1
- 主表 T11 備注移除「彙整 T07 全員心得」

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/工作分配.xlsx
+++ b/工作分配.xlsx
@@ -391,7 +391,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -603,6 +603,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -1041,7 +1044,7 @@
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>開發環境 + Docker Compose（db 服務先起）</t>
+          <t>開發環境 + Docker Compose（api/worker；DB 用 Neon 雲端）</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
@@ -1074,18 +1077,16 @@
       </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>docker-compose 能起 db</t>
-        </is>
-      </c>
-      <c r="M5" s="14" t="inlineStr">
+          <t>Compose(api/worker) 起得來 + 能連上 Neon</t>
+        </is>
+      </c>
+      <c r="M5" s="79" t="inlineStr">
         <is>
           <t>• 環境：裝 Docker Desktop，docker compose version 可跑
-• 檔案：寫 docker-compose.yml 的 db 服務，image pgvector/pgvector:pg16
-• 先做：只起 db（compose up -d db），能用 DBeaver/psql 連上就算過
-• 存哪：DB 資料掛 volume，容器重建資料不消失
-• 秘密：DB 密碼放 .env（複製 .env.example），別寫死
-• ★ 這步是全隊地基：你做完別人才連得上資料庫
-• ★ 關鍵節點：完成後與 Haoche 一起驗收再通知下游</t>
+• DB：不起本地 db 容器，改連 Neon 雲端 Postgres——先在 Neon 建專案，連線字串放 .env(DATABASE_URL)，全隊共用同一個庫
+• 檔案：docker-compose.yml 只含 api + worker 兩服務（原 db 那格移除）
+• 先做：能連上 Neon（DBeaver/psql 用連線字串連通）+ api 容器起得來就算過
+• 好處：不用每人各起本地 db、資料共享；排程只在整合/demo 期跑，Neon 免費層 CU-hrs 夠</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1108,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>PostgreSQL + pgvector 建置 + init.sql</t>
+          <t>Neon 建庫 + pgvector + init.sql</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -1140,16 +1141,16 @@
       </c>
       <c r="L6" s="9" t="inlineStr">
         <is>
-          <t>可連線的向量資料庫</t>
-        </is>
-      </c>
-      <c r="M6" s="14" t="inlineStr">
-        <is>
-          <t>• 環境：T01 的 db 容器要先起來
-• 檔案：infra_Nash/postgres/init.sql 寫 CREATE EXTENSION vector;
+          <t>Neon 上可連線、pgvector 就緒的向量庫</t>
+        </is>
+      </c>
+      <c r="M6" s="79" t="inlineStr">
+        <is>
+          <t>• 環境：Neon 專案已建、連線字串就緒（T01）
+• 先確認：Neon 的 pgvector 擴充是否支援 vector(1024)（未驗證，動手前查官方）
+• 檔案：infra_Nash/postgres/init.sql 寫 CREATE EXTENSION vector;（在 Neon 上跑）
 • 注意：向量欄位維度 = 1024（BGE-M3）
-• 驗證：能建一張含 vector(1024) 的測試表
-• ★ 關鍵節點：完成後與 Haoche 一起驗收再通知下游</t>
+• 驗證：能在 Neon 建一張含 vector(1024) 的測試表</t>
         </is>
       </c>
     </row>
@@ -1656,7 +1657,7 @@
       <c r="M14" s="10" t="inlineStr">
         <is>
           <t>• ★ 環境：需 db(T01)+events 表(T03)；模型檔放 data/models/（別進 git）
-• 前置：彙整 T07 全員心得
+• BGE-M3 已定案（Timyo dedup.py）；T07 全員實驗已取消
 • 定案：模型 / 維度1024 / 前處理 / 去重閾值 一組寫死
 • 檔案：backend/app/pipeline/embedding_Timyo/bge_m3.py
 • 存哪：讀 articles(pending) → 算向量 → 寫 events.embedding → status=vectorized</t>
@@ -2877,7 +2878,7 @@
       </c>
       <c r="B5" s="32" t="inlineStr">
         <is>
-          <t>開發環境 + Docker Compose（db 服務先起）</t>
+          <t>開發環境 + Docker Compose（api/worker；DB 用 Neon 雲端）</t>
         </is>
       </c>
       <c r="C5" s="33" t="inlineStr">
@@ -2918,7 +2919,7 @@
       </c>
       <c r="B6" s="28" t="inlineStr">
         <is>
-          <t>PostgreSQL + pgvector 建置 + init.sql</t>
+          <t>Neon 建庫 + pgvector + init.sql</t>
         </is>
       </c>
       <c r="C6" s="33" t="inlineStr">
@@ -4005,11 +4006,11 @@
         </is>
       </c>
       <c r="C3" s="65" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D3" s="28" t="inlineStr">
         <is>
-          <t>T01、T02、T03、T04、T07、T17、T19、T20、T25、T26、T27</t>
+          <t>T01、T02、T03、T04、T17、T19、T20、T25、T26、T27</t>
         </is>
       </c>
     </row>
@@ -4025,11 +4026,11 @@
         </is>
       </c>
       <c r="C4" s="65" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D4" s="28" t="inlineStr">
         <is>
-          <t>T05、T06、T07、T10、T20、T21、T25、T26、T27</t>
+          <t>T05、T06、T10、T20、T21、T25、T26、T27</t>
         </is>
       </c>
     </row>
@@ -4045,11 +4046,11 @@
         </is>
       </c>
       <c r="C5" s="65" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D5" s="28" t="inlineStr">
         <is>
-          <t>T01、T07、T11、T12、T20、T23、T26、T27</t>
+          <t>T01、T11、T12、T20、T23、T26、T27</t>
         </is>
       </c>
     </row>
@@ -4065,11 +4066,11 @@
         </is>
       </c>
       <c r="C6" s="65" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D6" s="28" t="inlineStr">
         <is>
-          <t>T07、T13、T14、T17、T20、T22、T23、T26、T27</t>
+          <t>T13、T14、T17、T20、T22、T23、T26、T27</t>
         </is>
       </c>
     </row>
@@ -4085,11 +4086,11 @@
         </is>
       </c>
       <c r="C7" s="65" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D7" s="28" t="inlineStr">
         <is>
-          <t>T03、T07、T09、T15、T16、T17、T20、T21、T24、T26、T27</t>
+          <t>T03、T09、T15、T16、T17、T20、T21、T24、T26、T27</t>
         </is>
       </c>
     </row>
@@ -4105,11 +4106,11 @@
         </is>
       </c>
       <c r="C8" s="65" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D8" s="28" t="inlineStr">
         <is>
-          <t>T04、T06、T07、T08、T18、T19、T20、T22、T26、T27</t>
+          <t>T04、T06、T08、T18、T19、T20、T22、T26、T27</t>
         </is>
       </c>
     </row>
@@ -4125,11 +4126,11 @@
         </is>
       </c>
       <c r="C9" s="65" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D9" s="28" t="inlineStr">
         <is>
-          <t>T00、T01、T02、T03、T04、T07、T19、T20、T25、T26、T27</t>
+          <t>T00、T01、T02、T03、T04、T19、T20、T25、T26、T27</t>
         </is>
       </c>
     </row>
@@ -4188,14 +4189,14 @@
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="74" t="inlineStr">
         <is>
-          <t>4. 高優先任務配置 2–3 人：地基(T01-04)、Embedding 實驗(T07 全員)、市場驗證(T17 三人)、端到端串接(T20)、收尾(T26 全員)。</t>
+          <t>4. 高優先任務配置 2–3 人：地基(T01-04)、市場驗證(T17 三人)、端到端串接(T20)、收尾(T26 全員)。</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="74" t="inlineStr">
         <is>
-          <t>5. 先地基後模組再整合：W1 打通環境/資料流並全員玩 Embedding；W2 核心模組並行；W3 整合、驗證、Demo。契約優先(T04)讓前端可先用 Mock 並行。</t>
+          <t>5. CSV 解耦並行：各模組用冻结樣本(接口=v2 契約)獨立開發、不等 DB，DB 整合集中後段。W1 地基+各線並行、W2 核心模組、W3(壓至 D10) 整合/驗證/串接；T26/27 收尾。契約優先(T04)+Mock 讓前端並行。</t>
         </is>
       </c>
     </row>

</xml_diff>